<commit_message>
Ohio's printed 2025 bracket bases are on record, inconsistency and all (#1317)
The 2025 IT 1040 booklet and R.C. 5747.02 print the 2025 brackets as
$342.00 plus 2.75% over $26,050 and $2,394.32 plus 3.125% over
$100,000. Those two figures do not agree with each other: $2,394.32 is
$360.69 (the 2024 base) + 2.75% x $73,950; $342.00 would give
$2,375.63. The inconsistency is Ohio's, and the scenarios use the
figures as published.

OH_edd.xml now carries both bases (oh_bracket_2_base, oh_bracket_3_base)
with that note in their comments, ready for the #1200 rebuild of OH_Tax,
which still does not read them; OH_02 and OH_03 carry the same note next
to the arithmetic that uses each base. Nothing computes differently.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9N1MFXbqHGQEJEf1KJJAQ
</commit_message>
<xml_diff>
--- a/sampleprojects/TaxReturn/excel/states/OH.xlsx
+++ b/sampleprojects/TaxReturn/excel/states/OH.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>DT: OH Tax</t>
   </si>
@@ -131,7 +131,7 @@
     <t>result</t>
   </si>
   <si>
-    <t>(11 attributes)</t>
+    <t>(13 attributes)</t>
   </si>
   <si>
     <t>oh_bracket_1_limit</t>
@@ -158,6 +158,15 @@
     <t>OH tax rate for bracket 1 - 0% (2025)</t>
   </si>
   <si>
+    <t>oh_bracket_2_base</t>
+  </si>
+  <si>
+    <t>342.0</t>
+  </si>
+  <si>
+    <t>OH 2025 tax at the bottom of bracket 2: $342.00 plus 2.75% of Ohio taxable income over $26,050, as the 2025 IT 1040 booklet (tax.ohio.gov) and R.C. 5747.02 print it. Ohio printed figures are inconsistent: the over-$100,000 base $2,394.32 is $360.69 (the 2024 base) + 2.75% x $73,950, not $342.00 + 2.75% x $73,950 = $2,375.63. The printed $342.00 is used as published (#1317).</t>
+  </si>
+  <si>
     <t>oh_bracket_2_limit</t>
   </si>
   <si>
@@ -174,6 +183,15 @@
   </si>
   <si>
     <t>OH tax rate for bracket 2 - 2.75% (2025)</t>
+  </si>
+  <si>
+    <t>oh_bracket_3_base</t>
+  </si>
+  <si>
+    <t>2394.32</t>
+  </si>
+  <si>
+    <t>OH 2025 tax at the bottom of bracket 3: $2,394.32 plus 3.125% of Ohio taxable income over $100,000, as the 2025 IT 1040 booklet and R.C. 5747.02 print it. $2,394.32 is consistent only with the 2024 bracket-2 base $360.69, not the 2025 $342.00 (see oh_bracket_2_base); the inconsistency is Ohio own figures (#1317).</t>
   </si>
   <si>
     <t>oh_bracket_3_rate</t>
@@ -1729,7 +1747,7 @@
         <v>8</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>8</v>
@@ -1738,7 +1756,7 @@
         <v>42</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>8</v>
@@ -1753,6 +1771,88 @@
         <v>8</v>
       </c>
       <c r="M14" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="M16" s="7" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>